<commit_message>
Feat: Performed Data Wrangling specifically remove duplicates and formatted data
</commit_message>
<xml_diff>
--- a/Excel/Section_2_Excel_Wrangling_Practice_File.xlsx
+++ b/Excel/Section_2_Excel_Wrangling_Practice_File.xlsx
@@ -1,20 +1,40 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sankp\Downloads\python\Data-Analysis-And-Dashboards\Excel\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F8149D0-B33D-43AD-885F-7CE063B06FA6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="EmployeeData" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="24">
   <si>
     <t>Full Name</t>
   </si>
@@ -83,16 +103,19 @@
   </si>
   <si>
     <t>HR</t>
+  </si>
+  <si>
+    <t>Name</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
+    <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -156,13 +179,21 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -200,7 +231,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -234,6 +265,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -268,9 +300,10 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -443,11 +476,22 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:J6"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="14.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.77734375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="18.109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.88671875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.77734375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="9" width="18.109375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="14.88671875" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:10">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -479,7 +523,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:10">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>10</v>
       </c>
@@ -508,7 +552,7 @@
         <v>45458</v>
       </c>
     </row>
-    <row r="3" spans="1:10">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>11</v>
       </c>
@@ -537,7 +581,7 @@
         <v>45461</v>
       </c>
     </row>
-    <row r="4" spans="1:10">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>12</v>
       </c>
@@ -566,7 +610,7 @@
         <v>45463</v>
       </c>
     </row>
-    <row r="5" spans="1:10">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>13</v>
       </c>
@@ -595,7 +639,7 @@
         <v>45468</v>
       </c>
     </row>
-    <row r="6" spans="1:10">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>14</v>
       </c>
@@ -622,6 +666,92 @@
       </c>
       <c r="I6" s="2">
         <v>45473</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1F806A16-830A-4D24-BE2F-7268C180ABEE}">
+  <dimension ref="A1:C6"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="14.33203125" hidden="1" customWidth="1"/>
+    <col min="2" max="2" width="14.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.77734375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B2" t="str">
+        <f>PROPER(TRIM(A2))</f>
+        <v>John Doe</v>
+      </c>
+      <c r="C2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B3" t="str">
+        <f t="shared" ref="B3:B6" si="0">PROPER(TRIM(A3))</f>
+        <v>Jane Smith</v>
+      </c>
+      <c r="C3" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4" t="str">
+        <f t="shared" si="0"/>
+        <v>Alice Johnson</v>
+      </c>
+      <c r="C4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>13</v>
+      </c>
+      <c r="B5" t="str">
+        <f t="shared" si="0"/>
+        <v>Bob Brown</v>
+      </c>
+      <c r="C5" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>14</v>
+      </c>
+      <c r="B6" t="str">
+        <f t="shared" si="0"/>
+        <v>Eva White</v>
+      </c>
+      <c r="C6" t="s">
+        <v>19</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Feat: Performed data wrangling and techniques
</commit_message>
<xml_diff>
--- a/Excel/Section_2_Excel_Wrangling_Practice_File.xlsx
+++ b/Excel/Section_2_Excel_Wrangling_Practice_File.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sankp\Downloads\python\Data-Analysis-And-Dashboards\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F8149D0-B33D-43AD-885F-7CE063B06FA6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{541FF7A4-7C97-483F-8874-77FF367C1030}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="EmployeeData" sheetId="1" r:id="rId1"/>
-    <sheet name="Sheet1" sheetId="2" r:id="rId2"/>
+    <sheet name="Sheet2" sheetId="3" r:id="rId2"/>
+    <sheet name="Sheet1" sheetId="2" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -34,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="36">
   <si>
     <t>Full Name</t>
   </si>
@@ -106,6 +107,42 @@
   </si>
   <si>
     <t>Name</t>
+  </si>
+  <si>
+    <t>Domain</t>
+  </si>
+  <si>
+    <t>Name-Left</t>
+  </si>
+  <si>
+    <t>Middle</t>
+  </si>
+  <si>
+    <t>john</t>
+  </si>
+  <si>
+    <t>example.com</t>
+  </si>
+  <si>
+    <t>jane</t>
+  </si>
+  <si>
+    <t xml:space="preserve">User Name </t>
+  </si>
+  <si>
+    <t>e@example.com</t>
+  </si>
+  <si>
+    <t>@example.com</t>
+  </si>
+  <si>
+    <t>alic</t>
+  </si>
+  <si>
+    <t>bob@</t>
+  </si>
+  <si>
+    <t>eva@</t>
   </si>
 </sst>
 </file>
@@ -115,7 +152,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
   </numFmts>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -131,6 +168,14 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -140,7 +185,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -163,18 +208,48 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -674,17 +749,117 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1F806A16-830A-4D24-BE2F-7268C180ABEE}">
-  <dimension ref="A1:C6"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{17B5EA57-C0E5-442E-853B-15E516D91227}">
+  <dimension ref="A1:C13"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="14.33203125" hidden="1" customWidth="1"/>
-    <col min="2" max="2" width="14.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17.77734375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.77734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B2">
+        <v>50000</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B3">
+        <v>60000</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B4">
+        <v>55000</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>22</v>
+      </c>
+      <c r="B5">
+        <v>45000</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>21</v>
+      </c>
+      <c r="B6">
+        <v>70000</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="C10" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="B11" t="s">
+        <v>20</v>
+      </c>
+      <c r="C11">
+        <v>105000</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="B12" t="s">
+        <v>21</v>
+      </c>
+      <c r="C12">
+        <v>130000</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="B13" t="s">
+        <v>22</v>
+      </c>
+      <c r="C13">
+        <v>45000</v>
+      </c>
+    </row>
+  </sheetData>
+  <dataConsolidate leftLabels="1" topLabels="1">
+    <dataRefs count="1">
+      <dataRef ref="A1:B6" sheet="Sheet2"/>
+    </dataRefs>
+  </dataConsolidate>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1F806A16-830A-4D24-BE2F-7268C180ABEE}">
+  <dimension ref="A1:J6"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="20.6640625" hidden="1" customWidth="1"/>
+    <col min="2" max="2" width="22.21875" customWidth="1"/>
+    <col min="3" max="3" width="17.77734375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.88671875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.6640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
@@ -693,8 +868,23 @@
       <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D1" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F1" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G1" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="H1" s="5" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>10</v>
       </c>
@@ -702,11 +892,35 @@
         <f>PROPER(TRIM(A2))</f>
         <v>John Doe</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="3" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D2" t="str">
+        <f>RIGHT(C2,11)</f>
+        <v>example.com</v>
+      </c>
+      <c r="E2" t="str">
+        <f>LEFT(B2,3)</f>
+        <v>Joh</v>
+      </c>
+      <c r="F2" t="str">
+        <f>MID(C2,6,7)</f>
+        <v>example</v>
+      </c>
+      <c r="G2" t="s">
+        <v>27</v>
+      </c>
+      <c r="H2" t="s">
+        <v>28</v>
+      </c>
+      <c r="I2" t="s">
+        <v>27</v>
+      </c>
+      <c r="J2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>11</v>
       </c>
@@ -714,11 +928,35 @@
         <f t="shared" ref="B3:B6" si="0">PROPER(TRIM(A3))</f>
         <v>Jane Smith</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C3" s="3" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D3" t="str">
+        <f t="shared" ref="D3:D6" si="1">RIGHT(C3,11)</f>
+        <v>example.com</v>
+      </c>
+      <c r="E3" t="str">
+        <f t="shared" ref="E3:E6" si="2">LEFT(B3,3)</f>
+        <v>Jan</v>
+      </c>
+      <c r="F3" t="str">
+        <f t="shared" ref="F3:F6" si="3">MID(C3,6,7)</f>
+        <v>example</v>
+      </c>
+      <c r="G3" t="s">
+        <v>29</v>
+      </c>
+      <c r="H3" t="s">
+        <v>28</v>
+      </c>
+      <c r="I3" t="s">
+        <v>29</v>
+      </c>
+      <c r="J3" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>12</v>
       </c>
@@ -726,11 +964,35 @@
         <f t="shared" si="0"/>
         <v>Alice Johnson</v>
       </c>
-      <c r="C4" t="s">
+      <c r="C4" s="3" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D4" t="str">
+        <f t="shared" si="1"/>
+        <v>example.com</v>
+      </c>
+      <c r="E4" t="str">
+        <f t="shared" si="2"/>
+        <v>Ali</v>
+      </c>
+      <c r="F4" t="str">
+        <f t="shared" si="3"/>
+        <v>@exampl</v>
+      </c>
+      <c r="G4" t="s">
+        <v>33</v>
+      </c>
+      <c r="H4" t="s">
+        <v>28</v>
+      </c>
+      <c r="I4" t="s">
+        <v>33</v>
+      </c>
+      <c r="J4" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>13</v>
       </c>
@@ -741,8 +1003,32 @@
       <c r="C5" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D5" t="str">
+        <f t="shared" si="1"/>
+        <v>example.com</v>
+      </c>
+      <c r="E5" t="str">
+        <f t="shared" si="2"/>
+        <v>Bob</v>
+      </c>
+      <c r="F5" t="str">
+        <f t="shared" si="3"/>
+        <v>xample.</v>
+      </c>
+      <c r="G5" t="s">
+        <v>34</v>
+      </c>
+      <c r="H5" t="s">
+        <v>28</v>
+      </c>
+      <c r="I5" t="s">
+        <v>34</v>
+      </c>
+      <c r="J5" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>14</v>
       </c>
@@ -753,8 +1039,38 @@
       <c r="C6" t="s">
         <v>19</v>
       </c>
+      <c r="D6" t="str">
+        <f t="shared" si="1"/>
+        <v>example.com</v>
+      </c>
+      <c r="E6" t="str">
+        <f t="shared" si="2"/>
+        <v>Eva</v>
+      </c>
+      <c r="F6" t="str">
+        <f t="shared" si="3"/>
+        <v>xample.</v>
+      </c>
+      <c r="G6" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="H6" t="s">
+        <v>28</v>
+      </c>
+      <c r="I6" t="s">
+        <v>35</v>
+      </c>
+      <c r="J6" t="s">
+        <v>28</v>
+      </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="C2" r:id="rId1" xr:uid="{BC1F0038-8235-423C-8850-418458BAF351}"/>
+    <hyperlink ref="C3" r:id="rId2" xr:uid="{1865092C-C14C-4137-8798-BF7A5CE963A2}"/>
+    <hyperlink ref="C4" r:id="rId3" xr:uid="{4D5C2709-37B2-48F1-B73E-66F56232E93A}"/>
+    <hyperlink ref="G6" r:id="rId4" xr:uid="{9B02BE12-8E67-47EF-8EC3-80B09FCF7547}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>